<commit_message>
Created UI files and their respective loaders in python
</commit_message>
<xml_diff>
--- a/client/gui/widget_action_spreadsheet.xlsx
+++ b/client/gui/widget_action_spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yahel\Desktop\Github Desktop Respositories\Stegastatter\client\gui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC4C38A-8CC2-4A29-8F3B-AA82FD920C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139E051E-7EFC-402B-9AF6-A46F9941FACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12435" yWindow="4260" windowWidth="21735" windowHeight="15330" xr2:uid="{AF7E1D43-0338-44DD-AECF-A2C317638C69}"/>
+    <workbookView xWindow="19425" yWindow="11385" windowWidth="17400" windowHeight="8805" xr2:uid="{AF7E1D43-0338-44DD-AECF-A2C317638C69}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Vessel Image Input File</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>All Decoding</t>
+  </si>
+  <si>
+    <t>V</t>
   </si>
 </sst>
 </file>
@@ -105,7 +108,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,6 +133,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -254,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -265,31 +280,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -632,14 +656,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FAF41C5-458C-4610-951D-BB1ED4E29DCA}">
-  <dimension ref="B2:I13"/>
+  <dimension ref="B1:I13"/>
   <sheetFormatPr defaultColWidth="16.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" customWidth="1"/>
     <col min="2" max="2" width="33.140625" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+    </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="2" t="s">
@@ -665,135 +705,135 @@
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="8"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="13"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="10"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="14"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="10"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="14"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="14"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="14"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="14"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="14"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="10"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="14"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="14"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="14"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="7"/>
       <c r="I13" s="15"/>
     </row>
   </sheetData>

</xml_diff>